<commit_message>
ajustar medidas com 0 na frente
</commit_message>
<xml_diff>
--- a/planilhas/outputs/Relatorio_Dominios_Ambiguos.xlsx
+++ b/planilhas/outputs/Relatorio_Dominios_Ambiguos.xlsx
@@ -88,7 +88,7 @@
     <t>TELHA FIBROCIM S/AMARELO 2,44X0,92X5MM - INFI INFIBRA</t>
   </si>
   <si>
-    <t>LAPIS CARPINTEIRO CX72PC IRWIN</t>
+    <t>LAPIS CARPINTEIRO CX 72 PC IRWIN</t>
   </si>
   <si>
     <t>DISCO FLAP CONICO 80 4,5X22 ZICORNIO BOSCH</t>
@@ -2752,10 +2752,10 @@
     <t>PARAFUSO ROSCA MAQUINA REDONDA C 3/16 X 1 JOMARCA</t>
   </si>
   <si>
-    <t>PARAFUSO ROSCA MAQUINA REDONDA C 3/16 X 1 1/2 JOMARC JOMARCA</t>
-  </si>
-  <si>
-    <t>PARAFUSO ROSCA MAQUINA REDONDA C 3/16 X 3 JOMARC JOMARCA</t>
+    <t>PARAFUSO ROSCA MAQUINA REDONDA C 3/16 X 1 1/2 JORMARCA JOMARCA</t>
+  </si>
+  <si>
+    <t>PARAFUSO ROSCA MAQUINA REDONDA C 3/16 X 3 JORMARCA JOMARCA</t>
   </si>
   <si>
     <t>PARAFUSO A/A CHATA PHILIPS 4,2 X 16 JOMARCA</t>
@@ -2812,7 +2812,7 @@
     <t>PARAFUSO FRANCES B 1/4 X 2</t>
   </si>
   <si>
-    <t>PARAFUSO ROSCA MAQUINA REDONDA C 3/16 X 2 JOMARC JOMARCA</t>
+    <t>PARAFUSO ROSCA MAQUINA REDONDA C 3/16 X 2 JORMARCA JOMARCA</t>
   </si>
   <si>
     <t>PARAFUSO SEXTAVADO FERRO B 5/16 X 1 1/2 JOMARCA</t>

</xml_diff>